<commit_message>
feat: centralize locators in CommonPaths, add All_Scenarios suite, and fix GST fetch wait
</commit_message>
<xml_diff>
--- a/TestData/UITestData.xlsx
+++ b/TestData/UITestData.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="36">
   <si>
     <t>Username</t>
   </si>
@@ -94,6 +94,36 @@
   </si>
   <si>
     <t>24AAICA0488M1ZF</t>
+  </si>
+  <si>
+    <t>Branch Sub-Type dropdown option</t>
+  </si>
+  <si>
+    <t>Accommodation</t>
+  </si>
+  <si>
+    <t>Airport</t>
+  </si>
+  <si>
+    <t>Fleet</t>
+  </si>
+  <si>
+    <t>Hub</t>
+  </si>
+  <si>
+    <t>Mini Hub</t>
+  </si>
+  <si>
+    <t>Office</t>
+  </si>
+  <si>
+    <t>Train</t>
+  </si>
+  <si>
+    <t>Virtual</t>
+  </si>
+  <si>
+    <t>Warehouse</t>
   </si>
 </sst>
 </file>
@@ -140,9 +170,12 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -470,10 +503,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.28515625" customWidth="1"/>
     <col min="2" max="2" width="18.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.42578125" customWidth="1"/>
     <col min="4" max="4" width="15.5703125" bestFit="1" customWidth="1"/>
@@ -486,9 +519,10 @@
     <col min="12" max="12" width="21" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="23.85546875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="32.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:15">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -531,8 +565,11 @@
       <c r="N1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="2" spans="1:14">
+      <c r="O1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -574,6 +611,54 @@
       </c>
       <c r="N2" t="s">
         <v>23</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15">
+      <c r="O3" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15">
+      <c r="O4" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15">
+      <c r="O5" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15">
+      <c r="O6" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15">
+      <c r="O7" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15">
+      <c r="O8" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15">
+      <c r="O9" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15">
+      <c r="O10" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15">
+      <c r="O11" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -581,6 +666,7 @@
     <hyperlink ref="F2" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat: add universal API Auto-Login Base, Postman-like VariableManager (pm), and stabilize Branch UI scenarios
</commit_message>
<xml_diff>
--- a/TestData/UITestData.xlsx
+++ b/TestData/UITestData.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
   </bookViews>
   <sheets>
     <sheet name="Credential" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="41">
   <si>
     <t>Username</t>
   </si>
@@ -24,9 +24,6 @@
     <t>Password</t>
   </si>
   <si>
-    <t>SONY</t>
-  </si>
-  <si>
     <t>Kuchbhi@123</t>
   </si>
   <si>
@@ -124,6 +121,24 @@
   </si>
   <si>
     <t>Warehouse</t>
+  </si>
+  <si>
+    <t>Ground+1</t>
+  </si>
+  <si>
+    <t>Ground+2</t>
+  </si>
+  <si>
+    <t>Ground+3</t>
+  </si>
+  <si>
+    <t>Ground+4</t>
+  </si>
+  <si>
+    <t>Branch Floor dropdown option</t>
+  </si>
+  <si>
+    <t>VIJAY</t>
   </si>
 </sst>
 </file>
@@ -487,10 +502,10 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>2</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -503,7 +518,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19.28515625" customWidth="1"/>
@@ -520,79 +535,84 @@
     <col min="13" max="13" width="23.85546875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="32.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="32" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:16">
       <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
         <v>4</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>5</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>6</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>8</v>
       </c>
-      <c r="F1" t="s">
-        <v>9</v>
-      </c>
       <c r="G1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I1" t="s">
+        <v>16</v>
+      </c>
+      <c r="J1" t="s">
         <v>17</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>18</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>19</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>20</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>21</v>
       </c>
-      <c r="N1" t="s">
-        <v>22</v>
-      </c>
       <c r="O1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15">
+        <v>25</v>
+      </c>
+      <c r="P1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16">
       <c r="A2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" t="s">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>25</v>
-      </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D2">
         <v>9237937388</v>
       </c>
       <c r="E2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I2">
         <v>1</v>
@@ -610,55 +630,70 @@
         <v>1</v>
       </c>
       <c r="N2" t="s">
+        <v>22</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16">
+      <c r="O3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="P3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16">
+      <c r="O4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="O2" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15">
-      <c r="O3" s="2" t="s">
+      <c r="P4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16">
+      <c r="O5" s="2" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="4" spans="1:15">
-      <c r="O4" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15">
-      <c r="O5" s="2" t="s">
+      <c r="P5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16">
+      <c r="O6" s="2" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="6" spans="1:15">
-      <c r="O6" s="2" t="s">
+      <c r="P6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16">
+      <c r="O7" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:15">
-      <c r="O7" s="2" t="s">
+    <row r="8" spans="1:16">
+      <c r="O8" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
-      <c r="O8" s="2" t="s">
+    <row r="9" spans="1:16">
+      <c r="O9" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:15">
-      <c r="O9" s="2" t="s">
+    <row r="10" spans="1:16">
+      <c r="O10" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
-      <c r="O10" s="2" t="s">
+    <row r="11" spans="1:16">
+      <c r="O11" s="2" t="s">
         <v>34</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15">
-      <c r="O11" s="2" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>